<commit_message>
updated process scheduling slides
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1222419-DE57-3349-B4A2-B90B4206F08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A6B1D4-F334-CE4C-AD96-AE0359B90184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="116">
   <si>
     <t>Lecture</t>
   </si>
@@ -381,6 +381,12 @@
   </si>
   <si>
     <t>should check cutting in the beginning If we are no longer pointing to Silberschatz, those instructions should go from the slides</t>
+  </si>
+  <si>
+    <t>If we are no longer pointing to Silberschatz, those instructions should go from the slides. Also, important update on slide 7, should re-make the video!</t>
+  </si>
+  <si>
+    <t>This video is to be redone too (priority)</t>
   </si>
 </sst>
 </file>
@@ -1346,7 +1352,7 @@
         <v>14</v>
       </c>
       <c r="I21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -1425,6 +1431,9 @@
       </c>
       <c r="H24" t="s">
         <v>14</v>
+      </c>
+      <c r="I24" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
polishing synchronization part 1
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A6B1D4-F334-CE4C-AD96-AE0359B90184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEDEB2F-FDD1-C348-B4E5-FB307DA68091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="118">
   <si>
     <t>Lecture</t>
   </si>
@@ -387,6 +387,12 @@
   </si>
   <si>
     <t>This video is to be redone too (priority)</t>
+  </si>
+  <si>
+    <t>Conceptual error in example, needs to be re-recorded!</t>
+  </si>
+  <si>
+    <t>Some slides changed, should re-record</t>
   </si>
 </sst>
 </file>
@@ -415,7 +421,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -425,6 +431,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -441,12 +453,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1646,6 +1659,9 @@
       <c r="H32" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I32" s="5" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
@@ -1698,7 +1714,9 @@
       <c r="H34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I34" s="1"/>
+      <c r="I34" s="5" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">

</xml_diff>